<commit_message>
Initial commit with MotorPH Payroll system
</commit_message>
<xml_diff>
--- a/src/MotorPH_Employee_Data.xlsx
+++ b/src/MotorPH_Employee_Data.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhoan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ba4fa9d75cca4aa9/Documents/Desktop/Investments/Documents/NetBeansProjects/MotorPHPayrollFixed/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5945D5BB-426E-4DEE-A75C-D2BB3C95F1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{5945D5BB-426E-4DEE-A75C-D2BB3C95F1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A882E90-B108-4601-92B3-C2D6BE596FA0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee Details" sheetId="1" r:id="rId1"/>
-    <sheet name="Attendance Record" sheetId="3" state="hidden" r:id="rId2"/>
+    <sheet name="Users" sheetId="4" r:id="rId2"/>
+    <sheet name="Attendance Record" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Users!$A$1:$C$35</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -32,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4787" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4892" uniqueCount="342">
   <si>
     <t>Employee #</t>
   </si>
@@ -811,313 +815,253 @@
     <t>Lim.Antonio</t>
   </si>
   <si>
-    <t>Lim.Antonio02</t>
-  </si>
-  <si>
-    <t>Aquino.Bianca Sofia</t>
-  </si>
-  <si>
-    <t>Aquino.Bianca Sofia03</t>
-  </si>
-  <si>
     <t>Reyes.Isabella</t>
-  </si>
-  <si>
-    <t>Reyes.Isabella04</t>
   </si>
   <si>
     <t>Hernandez.Eduard</t>
   </si>
   <si>
-    <t>Hernandez.Eduard05</t>
-  </si>
-  <si>
-    <t>Villanueva.Andrea Mae</t>
-  </si>
-  <si>
-    <t>Villanueva.Andrea Mae06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Jose.Brad </t>
-  </si>
-  <si>
-    <t>San Jose.Brad 07</t>
-  </si>
-  <si>
     <t>Romualdez.Alice</t>
-  </si>
-  <si>
-    <t>Romualdez.Alice08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atienza.Rosie </t>
-  </si>
-  <si>
-    <t>Atienza.Rosie 09</t>
   </si>
   <si>
     <t>Alvaro.Roderick</t>
   </si>
   <si>
-    <t>Alvaro.Roderick010</t>
-  </si>
-  <si>
     <t>Salcedo.Anthony</t>
-  </si>
-  <si>
-    <t>Salcedo.Anthony011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lopez.Josie </t>
-  </si>
-  <si>
-    <t>Lopez.Josie 012</t>
   </si>
   <si>
     <t>Farala.Martha</t>
   </si>
   <si>
-    <t>Farala.Martha013</t>
-  </si>
-  <si>
     <t>Martinez.Leila</t>
-  </si>
-  <si>
-    <t>Martinez.Leila014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Romualdez.Fredrick </t>
-  </si>
-  <si>
-    <t>Romualdez.Fredrick 015</t>
   </si>
   <si>
     <t>Mata.Christian</t>
   </si>
   <si>
-    <t>Mata.Christian016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De Leon.Selena </t>
-  </si>
-  <si>
-    <t>De Leon.Selena 017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Jose.Allison </t>
-  </si>
-  <si>
-    <t>San Jose.Allison 018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rosario.Cydney </t>
-  </si>
-  <si>
-    <t>Rosario.Cydney 019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bautista.Mark </t>
-  </si>
-  <si>
-    <t>Bautista.Mark 020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lazaro.Darlene </t>
-  </si>
-  <si>
-    <t>Lazaro.Darlene 021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delos Santos.Kolby </t>
-  </si>
-  <si>
-    <t>Delos Santos.Kolby 022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santos.Vella </t>
-  </si>
-  <si>
-    <t>Santos.Vella 023</t>
-  </si>
-  <si>
-    <t>Del Rosario.Tomas</t>
-  </si>
-  <si>
-    <t>Del Rosario.Tomas024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tolentino.Jacklyn </t>
-  </si>
-  <si>
-    <t>Tolentino.Jacklyn 025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gutierrez.Percival </t>
-  </si>
-  <si>
-    <t>Gutierrez.Percival 026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manalaysay.Garfield </t>
-  </si>
-  <si>
-    <t>Manalaysay.Garfield 027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Villegas.Lizeth </t>
-  </si>
-  <si>
-    <t>Villegas.Lizeth 028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ramos.Carol </t>
-  </si>
-  <si>
-    <t>Ramos.Carol 029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maceda.Emelia </t>
-  </si>
-  <si>
-    <t>Maceda.Emelia 030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aguilar.Delia </t>
-  </si>
-  <si>
-    <t>Aguilar.Delia 031</t>
-  </si>
-  <si>
-    <t>Castro.John Rafael</t>
-  </si>
-  <si>
-    <t>Castro.John Rafael032</t>
-  </si>
-  <si>
-    <t>Martinez.Carlos Ian</t>
-  </si>
-  <si>
-    <t>Martinez.Carlos Ian033</t>
-  </si>
-  <si>
     <t>Santos.Beatriz</t>
-  </si>
-  <si>
-    <t>Santos.Beatriz034</t>
-  </si>
-  <si>
-    <t>Garcia.ManuelIII</t>
-  </si>
-  <si>
-    <t>Garcia.ManuelIII01</t>
-  </si>
-  <si>
-    <t>Full Name</t>
   </si>
   <si>
     <t>First Time Login</t>
   </si>
   <si>
-    <t>Garcia Manuel III</t>
+    <t>Role</t>
   </si>
   <si>
-    <t>Lim Antonio</t>
+    <t>Department</t>
   </si>
   <si>
-    <t>Aquino Bianca Sofia</t>
+    <t>Garcia.Manuel</t>
   </si>
   <si>
-    <t>Reyes Isabella</t>
+    <t>ADMIN</t>
   </si>
   <si>
-    <t>Hernandez Eduard</t>
+    <t>Executive</t>
   </si>
   <si>
-    <t>Villanueva Andrea Mae</t>
+    <t>Aquino.Bianca</t>
   </si>
   <si>
-    <t xml:space="preserve">San Jose Brad </t>
+    <t>IT</t>
   </si>
   <si>
-    <t>Romualdez Alice</t>
+    <t>Villanueva.Andrea</t>
   </si>
   <si>
-    <t xml:space="preserve">Atienza Rosie </t>
+    <t>SUPERVISOR</t>
   </si>
   <si>
-    <t>Alvaro Roderick</t>
+    <t>HR</t>
   </si>
   <si>
-    <t>Salcedo Anthony</t>
+    <t>EMPLOYEE</t>
   </si>
   <si>
-    <t xml:space="preserve">Lopez Josie </t>
+    <t>Accounting</t>
   </si>
   <si>
-    <t>Farala Martha</t>
+    <t>Payroll</t>
   </si>
   <si>
-    <t>Martinez Leila</t>
+    <t>PAYROLL</t>
   </si>
   <si>
-    <t xml:space="preserve">Romualdez Fredrick </t>
+    <t>Account</t>
   </si>
   <si>
-    <t>Mata Christian</t>
+    <t>DelRosario.Tomas</t>
   </si>
   <si>
-    <t xml:space="preserve">De Leon Selena </t>
+    <t>Castro.John</t>
   </si>
   <si>
-    <t xml:space="preserve">San Jose Allison </t>
+    <t>Sales</t>
   </si>
   <si>
-    <t xml:space="preserve">Rosario Cydney </t>
+    <t>Martinez.Carlos</t>
   </si>
   <si>
-    <t xml:space="preserve">Bautista Mark </t>
+    <t>Logistics</t>
   </si>
   <si>
-    <t xml:space="preserve">Lazaro Darlene </t>
+    <t>Customer Service</t>
   </si>
   <si>
-    <t xml:space="preserve">Delos Santos Kolby </t>
+    <t>Garcia.Manuel123</t>
   </si>
   <si>
-    <t xml:space="preserve">Santos Vella </t>
+    <t>Lim.Antonio123</t>
   </si>
   <si>
-    <t>Del Rosario Tomas</t>
+    <t>Aquino.Bianca123</t>
   </si>
   <si>
-    <t xml:space="preserve">Tolentino Jacklyn </t>
+    <t>Reyes.Isabella123</t>
   </si>
   <si>
-    <t xml:space="preserve">Gutierrez Percival </t>
+    <t>Hernandez.Eduard123</t>
   </si>
   <si>
-    <t xml:space="preserve">Manalaysay Garfield </t>
+    <t>Villanueva.Andrea123</t>
   </si>
   <si>
-    <t xml:space="preserve">Villegas Lizeth </t>
+    <t>Romualdez.Alice123</t>
   </si>
   <si>
-    <t xml:space="preserve">Ramos Carol </t>
+    <t>Alvaro.Roderick123</t>
   </si>
   <si>
-    <t xml:space="preserve">Maceda Emelia </t>
+    <t>Salcedo.Anthony123</t>
   </si>
   <si>
-    <t xml:space="preserve">Aguilar Delia </t>
+    <t>Farala.Martha123</t>
   </si>
   <si>
-    <t>Castro John Rafael</t>
+    <t>Martinez.Leila123</t>
   </si>
   <si>
-    <t>Martinez Carlos Ian</t>
+    <t>Mata.Christian123</t>
   </si>
   <si>
-    <t>Santos Beatriz</t>
+    <t>DelRosario.Tomas123</t>
+  </si>
+  <si>
+    <t>Castro.John123</t>
+  </si>
+  <si>
+    <t>Martinez.Carlos123</t>
+  </si>
+  <si>
+    <t>Santos.Beatriz123</t>
+  </si>
+  <si>
+    <t>SanJose.Brad123</t>
+  </si>
+  <si>
+    <t>Atienza.Rosie123</t>
+  </si>
+  <si>
+    <t>Lopez.Josie123</t>
+  </si>
+  <si>
+    <t>Romualdez.Fredrick123</t>
+  </si>
+  <si>
+    <t>DeLeon.Selena123</t>
+  </si>
+  <si>
+    <t>SanJose.Allison123</t>
+  </si>
+  <si>
+    <t>Rosario.Cydney123</t>
+  </si>
+  <si>
+    <t>Bautista.Mark123</t>
+  </si>
+  <si>
+    <t>Lazaro.Darlene123</t>
+  </si>
+  <si>
+    <t>DelosSantos.Kolby123</t>
+  </si>
+  <si>
+    <t>Santos.Vella123</t>
+  </si>
+  <si>
+    <t>Tolentino.Jacklyn123</t>
+  </si>
+  <si>
+    <t>Gutierrez.Percival123</t>
+  </si>
+  <si>
+    <t>Manalaysay.Garfield123</t>
+  </si>
+  <si>
+    <t>Villegas.Lizeth123</t>
+  </si>
+  <si>
+    <t>Ramos.Carol123</t>
+  </si>
+  <si>
+    <t>Maceda.Emelia123</t>
+  </si>
+  <si>
+    <t>Aguilar.Delia123</t>
+  </si>
+  <si>
+    <t>SanJose.Brad</t>
+  </si>
+  <si>
+    <t>Atienza.Rosie</t>
+  </si>
+  <si>
+    <t>Lopez.Josie</t>
+  </si>
+  <si>
+    <t>Romualdez.Fredrick</t>
+  </si>
+  <si>
+    <t>DeLeon.Selena</t>
+  </si>
+  <si>
+    <t>SanJose.Allison</t>
+  </si>
+  <si>
+    <t>Rosario.Cydney</t>
+  </si>
+  <si>
+    <t>Bautista.Mark</t>
+  </si>
+  <si>
+    <t>Lazaro.Darlene</t>
+  </si>
+  <si>
+    <t>DelosSantos.Kolby</t>
+  </si>
+  <si>
+    <t>Santos.Vella</t>
+  </si>
+  <si>
+    <t>Tolentino.Jacklyn</t>
+  </si>
+  <si>
+    <t>Gutierrez.Percival</t>
+  </si>
+  <si>
+    <t>Manalaysay.Garfield</t>
+  </si>
+  <si>
+    <t>Villegas.Lizeth</t>
+  </si>
+  <si>
+    <t>Ramos.Carol</t>
+  </si>
+  <si>
+    <t>Maceda.Emelia</t>
+  </si>
+  <si>
+    <t>Aguilar.Delia</t>
   </si>
 </sst>
 </file>
@@ -1189,7 +1133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1219,22 +1163,118 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA5A5A5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA5A5A5"/>
+      </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FFA5A5A5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA5A5A5"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFA5A5A5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA5A5A5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF999999"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FFA5A5A5"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFA5A5A5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA5A5A5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FFBFBFBF"/>
       </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA5A5A5"/>
+      </left>
+      <right/>
       <top/>
+      <bottom style="thin">
+        <color rgb="FFA5A5A5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFA5A5A5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA5A5A5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA5A5A5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFA5A5A5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA5A5A5"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1242,7 +1282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1259,55 +1299,138 @@
     <xf numFmtId="20" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1324,6 +1447,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1546,2559 +1673,2561 @@
     <col min="17" max="17" width="11" customWidth="1"/>
     <col min="18" max="18" width="13.33203125" customWidth="1"/>
     <col min="19" max="19" width="12.33203125" customWidth="1"/>
-    <col min="21" max="21" width="21.5546875" customWidth="1"/>
+    <col min="20" max="20" width="20.109375" style="50" customWidth="1"/>
+    <col min="21" max="21" width="21.5546875" style="50" customWidth="1"/>
+    <col min="22" max="23" width="14.44140625" style="50"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="30" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="R1" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="U1" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="V1" s="23" t="s">
-        <v>326</v>
-      </c>
-      <c r="W1" s="23" t="s">
-        <v>327</v>
+      <c r="U1" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="V1" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11">
-        <v>1</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="15">
+        <v>10001</v>
+      </c>
+      <c r="B2" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="17">
         <v>30600</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="14">
+      <c r="H2" s="19">
         <v>820126853951</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="14">
+      <c r="J2" s="19">
         <v>691295330870</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="16">
+      <c r="N2" s="21">
         <v>90000</v>
       </c>
-      <c r="O2" s="16">
+      <c r="O2" s="21">
         <v>1500</v>
       </c>
-      <c r="P2" s="16">
+      <c r="P2" s="21">
         <v>2000</v>
       </c>
-      <c r="Q2" s="16">
+      <c r="Q2" s="21">
         <v>1000</v>
       </c>
-      <c r="R2" s="16">
+      <c r="R2" s="21">
         <f t="shared" ref="R2:R35" si="0">N2/2</f>
         <v>45000</v>
       </c>
-      <c r="S2" s="17">
+      <c r="S2" s="22">
         <f t="shared" ref="S2:S35" si="1">(N2/21)/8</f>
         <v>535.71428571428567</v>
       </c>
-      <c r="T2" s="18" t="s">
-        <v>324</v>
-      </c>
-      <c r="U2" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="V2" t="s">
-        <v>328</v>
-      </c>
-      <c r="W2" t="b">
+      <c r="T2" s="49" t="s">
+        <v>271</v>
+      </c>
+      <c r="U2" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="V2" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="W2" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11">
-        <v>2</v>
-      </c>
-      <c r="B3" s="12" t="s">
+      <c r="A3" s="15">
+        <v>10002</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="17">
         <v>32313</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="14">
+      <c r="H3" s="19">
         <v>331735646338</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="19">
         <v>663904995411</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="K3" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="12" t="s">
+      <c r="L3" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="N3" s="16">
+      <c r="N3" s="21">
         <v>60000</v>
       </c>
-      <c r="O3" s="16">
+      <c r="O3" s="21">
         <v>1500</v>
       </c>
-      <c r="P3" s="16">
+      <c r="P3" s="21">
         <v>2000</v>
       </c>
-      <c r="Q3" s="16">
+      <c r="Q3" s="21">
         <v>1000</v>
       </c>
-      <c r="R3" s="16">
+      <c r="R3" s="21">
         <f t="shared" si="0"/>
         <v>30000</v>
       </c>
-      <c r="S3" s="17">
+      <c r="S3" s="22">
         <f t="shared" si="1"/>
         <v>357.14285714285717</v>
       </c>
-      <c r="T3" s="19" t="s">
+      <c r="T3" s="50" t="s">
         <v>258</v>
       </c>
-      <c r="U3" s="19" t="s">
-        <v>259</v>
-      </c>
-      <c r="V3" t="s">
-        <v>329</v>
-      </c>
-      <c r="W3" t="b">
+      <c r="U3" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="V3" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="W3" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11">
-        <v>3</v>
-      </c>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="15">
+        <v>10003</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="17">
         <v>32724</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="19">
         <v>177451189665</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="14">
+      <c r="J4" s="19">
         <v>171519773969</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="K4" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="L4" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="N4" s="16">
+      <c r="N4" s="21">
         <v>60000</v>
       </c>
-      <c r="O4" s="16">
+      <c r="O4" s="21">
         <v>1500</v>
       </c>
-      <c r="P4" s="16">
+      <c r="P4" s="21">
         <v>2000</v>
       </c>
-      <c r="Q4" s="16">
+      <c r="Q4" s="21">
         <v>1000</v>
       </c>
-      <c r="R4" s="16">
+      <c r="R4" s="21">
         <f t="shared" si="0"/>
         <v>30000</v>
       </c>
-      <c r="S4" s="17">
+      <c r="S4" s="22">
         <f t="shared" si="1"/>
         <v>357.14285714285717</v>
       </c>
-      <c r="T4" s="19" t="s">
-        <v>260</v>
-      </c>
-      <c r="U4" s="19" t="s">
-        <v>261</v>
-      </c>
-      <c r="V4" t="s">
-        <v>330</v>
-      </c>
-      <c r="W4" t="b">
+      <c r="T4" s="49" t="s">
+        <v>274</v>
+      </c>
+      <c r="U4" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="V4" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="W4" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
-        <v>4</v>
-      </c>
-      <c r="B5" s="12" t="s">
+      <c r="A5" s="25">
+        <v>10004</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="17">
         <v>34501</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="19">
         <v>341911411254</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="14">
+      <c r="J5" s="19">
         <v>416946776041</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K5" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L5" s="12" t="s">
+      <c r="L5" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="M5" s="15" t="s">
+      <c r="M5" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="N5" s="16">
+      <c r="N5" s="21">
         <v>60000</v>
       </c>
-      <c r="O5" s="16">
+      <c r="O5" s="21">
         <v>1500</v>
       </c>
-      <c r="P5" s="16">
+      <c r="P5" s="21">
         <v>2000</v>
       </c>
-      <c r="Q5" s="16">
+      <c r="Q5" s="21">
         <v>1000</v>
       </c>
-      <c r="R5" s="16">
+      <c r="R5" s="21">
         <f t="shared" si="0"/>
         <v>30000</v>
       </c>
-      <c r="S5" s="17">
+      <c r="S5" s="22">
         <f t="shared" si="1"/>
         <v>357.14285714285717</v>
       </c>
-      <c r="T5" s="19" t="s">
-        <v>262</v>
-      </c>
-      <c r="U5" s="19" t="s">
-        <v>263</v>
-      </c>
-      <c r="V5" t="s">
-        <v>331</v>
-      </c>
-      <c r="W5" t="b">
+      <c r="T5" s="50" t="s">
+        <v>259</v>
+      </c>
+      <c r="U5" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="V5" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="W5" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11">
-        <v>5</v>
-      </c>
-      <c r="B6" s="12" t="s">
+      <c r="A6" s="25">
+        <v>10005</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="17">
         <v>32774</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="19">
         <v>957436191812</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="I6" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="19">
         <v>952347222457</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="L6" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M6" s="15" t="s">
+      <c r="M6" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="N6" s="16">
+      <c r="N6" s="21">
         <v>52670</v>
       </c>
-      <c r="O6" s="16">
+      <c r="O6" s="21">
         <v>1500</v>
       </c>
-      <c r="P6" s="16">
+      <c r="P6" s="21">
         <v>1000</v>
       </c>
-      <c r="Q6" s="16">
+      <c r="Q6" s="21">
         <v>1000</v>
       </c>
-      <c r="R6" s="16">
+      <c r="R6" s="21">
         <f t="shared" si="0"/>
         <v>26335</v>
       </c>
-      <c r="S6" s="17">
+      <c r="S6" s="26">
         <f t="shared" si="1"/>
         <v>313.51190476190476</v>
       </c>
-      <c r="T6" s="19" t="s">
-        <v>264</v>
-      </c>
-      <c r="U6" s="19" t="s">
-        <v>265</v>
-      </c>
-      <c r="V6" t="s">
-        <v>332</v>
-      </c>
-      <c r="W6" t="b">
+      <c r="T6" s="50" t="s">
+        <v>260</v>
+      </c>
+      <c r="U6" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="V6" s="49" t="s">
+        <v>275</v>
+      </c>
+      <c r="W6" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11">
-        <v>6</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="25">
+        <v>10006</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="17">
         <v>32187</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="19">
         <v>382189453145</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="19">
         <v>441093369646</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="M7" s="15" t="s">
+      <c r="M7" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="N7" s="16">
+      <c r="N7" s="21">
         <v>52670</v>
       </c>
-      <c r="O7" s="16">
+      <c r="O7" s="21">
         <v>1500</v>
       </c>
-      <c r="P7" s="16">
+      <c r="P7" s="21">
         <v>1000</v>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="21">
         <v>1000</v>
       </c>
-      <c r="R7" s="16">
+      <c r="R7" s="21">
         <f t="shared" si="0"/>
         <v>26335</v>
       </c>
-      <c r="S7" s="17">
+      <c r="S7" s="27">
         <f t="shared" si="1"/>
         <v>313.51190476190476</v>
       </c>
-      <c r="T7" s="19" t="s">
-        <v>266</v>
-      </c>
-      <c r="U7" s="19" t="s">
-        <v>267</v>
-      </c>
-      <c r="V7" t="s">
-        <v>333</v>
-      </c>
-      <c r="W7" t="b">
+      <c r="T7" s="49" t="s">
+        <v>276</v>
+      </c>
+      <c r="U7" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V7" s="49" t="s">
+        <v>278</v>
+      </c>
+      <c r="W7" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11">
-        <v>7</v>
-      </c>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="25">
+        <v>10007</v>
+      </c>
+      <c r="B8" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="29">
         <v>35139</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="30">
         <v>239192926939</v>
       </c>
-      <c r="I8" s="14" t="s">
+      <c r="I8" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="30">
         <v>210850209964</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="K8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L8" s="12" t="s">
+      <c r="L8" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="M8" s="15" t="s">
+      <c r="M8" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="N8" s="16">
+      <c r="N8" s="32">
         <v>42975</v>
       </c>
-      <c r="O8" s="16">
+      <c r="O8" s="32">
         <v>1500</v>
       </c>
-      <c r="P8" s="16">
+      <c r="P8" s="32">
         <v>800</v>
       </c>
-      <c r="Q8" s="16">
+      <c r="Q8" s="33">
         <v>800</v>
       </c>
-      <c r="R8" s="16">
+      <c r="R8" s="32">
         <f t="shared" si="0"/>
         <v>21487.5</v>
       </c>
-      <c r="S8" s="17">
+      <c r="S8" s="27">
         <f t="shared" si="1"/>
         <v>255.80357142857142</v>
       </c>
-      <c r="T8" s="19" t="s">
-        <v>268</v>
-      </c>
-      <c r="U8" s="19" t="s">
-        <v>269</v>
-      </c>
-      <c r="V8" t="s">
-        <v>334</v>
-      </c>
-      <c r="W8" t="b">
+      <c r="T8" s="49" t="s">
+        <v>324</v>
+      </c>
+      <c r="U8" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V8" s="49" t="s">
+        <v>278</v>
+      </c>
+      <c r="W8" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11">
-        <v>8</v>
-      </c>
-      <c r="B9" s="12" t="s">
+      <c r="A9" s="25">
+        <v>10008</v>
+      </c>
+      <c r="B9" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="29">
         <v>33738</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="14">
+      <c r="H9" s="30">
         <v>545652640232</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="30">
         <v>211385556888</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="K9" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="12" t="s">
+      <c r="L9" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="M9" s="15" t="s">
+      <c r="M9" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="N9" s="16">
+      <c r="N9" s="32">
         <v>22500</v>
       </c>
-      <c r="O9" s="16">
+      <c r="O9" s="32">
         <v>1500</v>
       </c>
-      <c r="P9" s="16">
+      <c r="P9" s="32">
         <v>500</v>
       </c>
-      <c r="Q9" s="16">
+      <c r="Q9" s="33">
         <v>500</v>
       </c>
-      <c r="R9" s="16">
+      <c r="R9" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S9" s="17">
+      <c r="S9" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T9" s="19" t="s">
-        <v>270</v>
-      </c>
-      <c r="U9" s="19" t="s">
-        <v>271</v>
-      </c>
-      <c r="V9" t="s">
-        <v>335</v>
-      </c>
-      <c r="W9" t="b">
+      <c r="T9" s="50" t="s">
+        <v>261</v>
+      </c>
+      <c r="U9" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V9" s="49" t="s">
+        <v>278</v>
+      </c>
+      <c r="W9" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11">
-        <v>9</v>
-      </c>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="34">
+        <v>10009</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="36">
         <v>17800</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="35" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="H10" s="14">
+      <c r="H10" s="37">
         <v>708988234853</v>
       </c>
-      <c r="I10" s="14" t="s">
+      <c r="I10" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="37">
         <v>260107732354</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="12" t="s">
+      <c r="L10" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="M10" s="15" t="s">
+      <c r="M10" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="N10" s="16">
+      <c r="N10" s="32">
         <v>22500</v>
       </c>
-      <c r="O10" s="16">
+      <c r="O10" s="32">
         <v>1500</v>
       </c>
-      <c r="P10" s="16">
+      <c r="P10" s="32">
         <v>500</v>
       </c>
-      <c r="Q10" s="16">
+      <c r="Q10" s="33">
         <v>500</v>
       </c>
-      <c r="R10" s="16">
+      <c r="R10" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S10" s="17">
+      <c r="S10" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T10" s="19" t="s">
-        <v>272</v>
-      </c>
-      <c r="U10" s="19" t="s">
-        <v>273</v>
-      </c>
-      <c r="V10" t="s">
-        <v>336</v>
-      </c>
-      <c r="W10" t="b">
+      <c r="T10" s="50" t="s">
+        <v>325</v>
+      </c>
+      <c r="U10" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V10" s="49" t="s">
+        <v>278</v>
+      </c>
+      <c r="W10" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="18">
+        <v>10010</v>
+      </c>
+      <c r="B11" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="17">
         <v>32232</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="H11" s="14">
+      <c r="H11" s="19">
         <v>578114853194</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="J11" s="14">
+      <c r="J11" s="19">
         <v>799254095212</v>
       </c>
-      <c r="K11" s="11" t="s">
+      <c r="K11" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="L11" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="M11" s="15" t="s">
+      <c r="M11" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="N11" s="16">
+      <c r="N11" s="21">
         <v>52670</v>
       </c>
-      <c r="O11" s="16">
+      <c r="O11" s="32">
         <v>1500</v>
       </c>
-      <c r="P11" s="16">
+      <c r="P11" s="21">
         <v>1000</v>
       </c>
-      <c r="Q11" s="16">
+      <c r="Q11" s="21">
         <v>1000</v>
       </c>
-      <c r="R11" s="16">
+      <c r="R11" s="32">
         <f t="shared" si="0"/>
         <v>26335</v>
       </c>
-      <c r="S11" s="17">
+      <c r="S11" s="27">
         <f t="shared" si="1"/>
         <v>313.51190476190476</v>
       </c>
-      <c r="T11" s="19" t="s">
-        <v>274</v>
-      </c>
-      <c r="U11" s="19" t="s">
-        <v>275</v>
-      </c>
-      <c r="V11" t="s">
-        <v>337</v>
-      </c>
-      <c r="W11" t="b">
+      <c r="T11" s="50" t="s">
+        <v>262</v>
+      </c>
+      <c r="U11" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V11" s="49" t="s">
+        <v>280</v>
+      </c>
+      <c r="W11" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11">
-        <v>11</v>
-      </c>
-      <c r="B12" s="12" t="s">
+      <c r="A12" s="39">
+        <v>10011</v>
+      </c>
+      <c r="B12" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="17">
         <v>34226</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="H12" s="14">
+      <c r="H12" s="19">
         <v>126445315651</v>
       </c>
-      <c r="I12" s="14" t="s">
+      <c r="I12" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="J12" s="14">
+      <c r="J12" s="19">
         <v>218002473454</v>
       </c>
-      <c r="K12" s="11" t="s">
+      <c r="K12" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="L12" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="M12" s="15" t="s">
+      <c r="M12" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="N12" s="16">
+      <c r="N12" s="21">
         <v>50825</v>
       </c>
-      <c r="O12" s="16">
+      <c r="O12" s="21">
         <v>1500</v>
       </c>
-      <c r="P12" s="16">
+      <c r="P12" s="21">
         <v>1000</v>
       </c>
-      <c r="Q12" s="16">
+      <c r="Q12" s="21">
         <v>1000</v>
       </c>
-      <c r="R12" s="16">
+      <c r="R12" s="40">
         <f t="shared" si="0"/>
         <v>25412.5</v>
       </c>
-      <c r="S12" s="17">
+      <c r="S12" s="27">
         <f t="shared" si="1"/>
         <v>302.52976190476193</v>
       </c>
-      <c r="T12" s="19" t="s">
-        <v>276</v>
-      </c>
-      <c r="U12" s="19" t="s">
+      <c r="T12" s="50" t="s">
+        <v>263</v>
+      </c>
+      <c r="U12" s="49" t="s">
         <v>277</v>
       </c>
-      <c r="V12" t="s">
-        <v>338</v>
-      </c>
-      <c r="W12" t="b">
+      <c r="V12" s="49" t="s">
+        <v>281</v>
+      </c>
+      <c r="W12" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
-        <v>12</v>
-      </c>
-      <c r="B13" s="12" t="s">
+      <c r="A13" s="25">
+        <v>10012</v>
+      </c>
+      <c r="B13" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="17">
         <v>31791</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="H13" s="14">
+      <c r="H13" s="19">
         <v>431709011012</v>
       </c>
-      <c r="I13" s="14" t="s">
+      <c r="I13" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="19">
         <v>113071293354</v>
       </c>
-      <c r="K13" s="11" t="s">
+      <c r="K13" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L13" s="12" t="s">
+      <c r="L13" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="M13" s="15" t="s">
+      <c r="M13" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="N13" s="16">
+      <c r="N13" s="21">
         <v>38475</v>
       </c>
-      <c r="O13" s="16">
+      <c r="O13" s="21">
         <v>1500</v>
       </c>
-      <c r="P13" s="16">
+      <c r="P13" s="21">
         <v>800</v>
       </c>
-      <c r="Q13" s="16">
+      <c r="Q13" s="21">
         <v>800</v>
       </c>
-      <c r="R13" s="16">
+      <c r="R13" s="40">
         <f t="shared" si="0"/>
         <v>19237.5</v>
       </c>
-      <c r="S13" s="17">
+      <c r="S13" s="27">
         <f t="shared" si="1"/>
         <v>229.01785714285714</v>
       </c>
-      <c r="T13" s="19" t="s">
-        <v>278</v>
-      </c>
-      <c r="U13" s="19" t="s">
-        <v>279</v>
-      </c>
-      <c r="V13" t="s">
-        <v>339</v>
-      </c>
-      <c r="W13" t="b">
+      <c r="T13" s="50" t="s">
+        <v>326</v>
+      </c>
+      <c r="U13" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V13" s="49" t="s">
+        <v>281</v>
+      </c>
+      <c r="W13" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11">
-        <v>13</v>
-      </c>
-      <c r="B14" s="12" t="s">
+      <c r="A14" s="25">
+        <v>10013</v>
+      </c>
+      <c r="B14" s="28" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="29">
         <v>15352</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="H14" s="14">
+      <c r="H14" s="30">
         <v>233693897247</v>
       </c>
-      <c r="I14" s="14" t="s">
+      <c r="I14" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="30">
         <v>631130283546</v>
       </c>
-      <c r="K14" s="11" t="s">
+      <c r="K14" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L14" s="12" t="s">
+      <c r="L14" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="M14" s="15" t="s">
+      <c r="M14" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="N14" s="16">
+      <c r="N14" s="32">
         <v>24000</v>
       </c>
-      <c r="O14" s="16">
+      <c r="O14" s="32">
         <v>1500</v>
       </c>
-      <c r="P14" s="16">
+      <c r="P14" s="32">
         <v>500</v>
       </c>
-      <c r="Q14" s="16">
+      <c r="Q14" s="33">
         <v>500</v>
       </c>
-      <c r="R14" s="16">
+      <c r="R14" s="32">
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="S14" s="17">
+      <c r="S14" s="27">
         <f t="shared" si="1"/>
         <v>142.85714285714286</v>
       </c>
-      <c r="T14" s="19" t="s">
-        <v>280</v>
-      </c>
-      <c r="U14" s="19" t="s">
+      <c r="T14" s="50" t="s">
+        <v>264</v>
+      </c>
+      <c r="U14" s="49" t="s">
+        <v>282</v>
+      </c>
+      <c r="V14" s="49" t="s">
         <v>281</v>
       </c>
-      <c r="V14" t="s">
-        <v>340</v>
-      </c>
-      <c r="W14" t="b">
+      <c r="W14" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="11">
-        <v>14</v>
-      </c>
-      <c r="B15" s="12" t="s">
+      <c r="A15" s="25">
+        <v>10014</v>
+      </c>
+      <c r="B15" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="29">
         <v>25760</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="28" t="s">
         <v>120</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="H15" s="14">
+      <c r="H15" s="30">
         <v>515741057496</v>
       </c>
-      <c r="I15" s="14" t="s">
+      <c r="I15" s="30" t="s">
         <v>123</v>
       </c>
-      <c r="J15" s="14">
+      <c r="J15" s="30">
         <v>101205445886</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="K15" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L15" s="12" t="s">
+      <c r="L15" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="M15" s="15" t="s">
+      <c r="M15" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="N15" s="16">
+      <c r="N15" s="32">
         <v>24000</v>
       </c>
-      <c r="O15" s="16">
+      <c r="O15" s="32">
         <v>1500</v>
       </c>
-      <c r="P15" s="16">
+      <c r="P15" s="32">
         <v>500</v>
       </c>
-      <c r="Q15" s="16">
+      <c r="Q15" s="33">
         <v>500</v>
       </c>
-      <c r="R15" s="16">
+      <c r="R15" s="32">
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="S15" s="17">
+      <c r="S15" s="27">
         <f t="shared" si="1"/>
         <v>142.85714285714286</v>
       </c>
-      <c r="T15" s="19" t="s">
+      <c r="T15" s="50" t="s">
+        <v>265</v>
+      </c>
+      <c r="U15" s="49" t="s">
         <v>282</v>
       </c>
-      <c r="U15" s="19" t="s">
-        <v>283</v>
-      </c>
-      <c r="V15" t="s">
-        <v>341</v>
-      </c>
-      <c r="W15" t="b">
+      <c r="V15" s="49" t="s">
+        <v>281</v>
+      </c>
+      <c r="W15" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="11">
-        <v>15</v>
-      </c>
-      <c r="B16" s="12" t="s">
+      <c r="A16" s="25">
+        <v>10015</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="17">
         <v>31116</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="H16" s="14">
+      <c r="H16" s="19">
         <v>308366860059</v>
       </c>
-      <c r="I16" s="14" t="s">
+      <c r="I16" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="14">
+      <c r="J16" s="19">
         <v>223057707853</v>
       </c>
-      <c r="K16" s="11" t="s">
+      <c r="K16" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L16" s="20" t="s">
+      <c r="L16" s="41" t="s">
         <v>129</v>
       </c>
-      <c r="M16" s="21" t="s">
+      <c r="M16" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="N16" s="16">
+      <c r="N16" s="21">
         <v>53500</v>
       </c>
-      <c r="O16" s="16">
+      <c r="O16" s="21">
         <v>1500</v>
       </c>
-      <c r="P16" s="16">
+      <c r="P16" s="21">
         <v>1000</v>
       </c>
-      <c r="Q16" s="16">
+      <c r="Q16" s="21">
         <v>1000</v>
       </c>
-      <c r="R16" s="16">
+      <c r="R16" s="40">
         <f t="shared" si="0"/>
         <v>26750</v>
       </c>
-      <c r="S16" s="17">
+      <c r="S16" s="27">
         <f t="shared" si="1"/>
         <v>318.45238095238096</v>
       </c>
-      <c r="T16" s="19" t="s">
-        <v>284</v>
-      </c>
-      <c r="U16" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="V16" t="s">
-        <v>342</v>
-      </c>
-      <c r="W16" t="b">
+      <c r="T16" s="50" t="s">
+        <v>327</v>
+      </c>
+      <c r="U16" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V16" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W16" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11">
-        <v>16</v>
-      </c>
-      <c r="B17" s="12" t="s">
+      <c r="A17" s="25">
+        <v>10016</v>
+      </c>
+      <c r="B17" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="17">
         <v>32071</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="H17" s="14">
+      <c r="H17" s="19">
         <v>824187961962</v>
       </c>
-      <c r="I17" s="14" t="s">
+      <c r="I17" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="J17" s="14">
+      <c r="J17" s="19">
         <v>631052853464</v>
       </c>
-      <c r="K17" s="11" t="s">
+      <c r="K17" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L17" s="12" t="s">
+      <c r="L17" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="M17" s="15" t="s">
+      <c r="M17" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="N17" s="16">
+      <c r="N17" s="21">
         <v>42975</v>
       </c>
-      <c r="O17" s="16">
+      <c r="O17" s="21">
         <v>1500</v>
       </c>
-      <c r="P17" s="16">
+      <c r="P17" s="21">
         <v>800</v>
       </c>
-      <c r="Q17" s="16">
+      <c r="Q17" s="21">
         <v>800</v>
       </c>
-      <c r="R17" s="16">
+      <c r="R17" s="40">
         <f t="shared" si="0"/>
         <v>21487.5</v>
       </c>
-      <c r="S17" s="17">
+      <c r="S17" s="27">
         <f t="shared" si="1"/>
         <v>255.80357142857142</v>
       </c>
-      <c r="T17" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="U17" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="V17" t="s">
-        <v>343</v>
-      </c>
-      <c r="W17" t="b">
+      <c r="T17" s="50" t="s">
+        <v>266</v>
+      </c>
+      <c r="U17" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V17" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W17" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11">
-        <v>17</v>
-      </c>
-      <c r="B18" s="12" t="s">
+      <c r="A18" s="25">
+        <v>10017</v>
+      </c>
+      <c r="B18" s="28" t="s">
         <v>138</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="29">
         <v>27445</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="H18" s="14">
+      <c r="H18" s="30">
         <v>587272469938</v>
       </c>
-      <c r="I18" s="14" t="s">
+      <c r="I18" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="J18" s="14">
+      <c r="J18" s="30">
         <v>719007608464</v>
       </c>
-      <c r="K18" s="11" t="s">
+      <c r="K18" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L18" s="12" t="s">
+      <c r="L18" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="M18" s="15" t="s">
+      <c r="M18" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="N18" s="16">
+      <c r="N18" s="32">
         <v>41850</v>
       </c>
-      <c r="O18" s="16">
+      <c r="O18" s="32">
         <v>1500</v>
       </c>
-      <c r="P18" s="16">
+      <c r="P18" s="32">
         <v>800</v>
       </c>
-      <c r="Q18" s="16">
+      <c r="Q18" s="33">
         <v>800</v>
       </c>
-      <c r="R18" s="16">
+      <c r="R18" s="32">
         <f t="shared" si="0"/>
         <v>20925</v>
       </c>
-      <c r="S18" s="17">
+      <c r="S18" s="27">
         <f t="shared" si="1"/>
         <v>249.10714285714286</v>
       </c>
-      <c r="T18" s="19" t="s">
-        <v>288</v>
-      </c>
-      <c r="U18" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="V18" t="s">
-        <v>344</v>
-      </c>
-      <c r="W18" t="b">
+      <c r="T18" s="49" t="s">
+        <v>328</v>
+      </c>
+      <c r="U18" s="49" t="s">
+        <v>277</v>
+      </c>
+      <c r="V18" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W18" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="11">
-        <v>18</v>
-      </c>
-      <c r="B19" s="12" t="s">
+      <c r="A19" s="25">
+        <v>10018</v>
+      </c>
+      <c r="B19" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="29">
         <v>31587</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="H19" s="14">
+      <c r="H19" s="30">
         <v>745148459521</v>
       </c>
-      <c r="I19" s="14" t="s">
+      <c r="I19" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="J19" s="14">
+      <c r="J19" s="30">
         <v>114901859343</v>
       </c>
-      <c r="K19" s="11" t="s">
+      <c r="K19" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L19" s="12" t="s">
+      <c r="L19" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M19" s="15" t="s">
+      <c r="M19" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N19" s="16">
+      <c r="N19" s="32">
         <v>22500</v>
       </c>
-      <c r="O19" s="16">
+      <c r="O19" s="32">
         <v>1500</v>
       </c>
-      <c r="P19" s="16">
+      <c r="P19" s="32">
         <v>500</v>
       </c>
-      <c r="Q19" s="16">
+      <c r="Q19" s="33">
         <v>500</v>
       </c>
-      <c r="R19" s="16">
+      <c r="R19" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S19" s="17">
+      <c r="S19" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T19" s="19" t="s">
-        <v>290</v>
-      </c>
-      <c r="U19" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="V19" t="s">
-        <v>345</v>
-      </c>
-      <c r="W19" t="b">
+      <c r="T19" s="49" t="s">
+        <v>329</v>
+      </c>
+      <c r="U19" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V19" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W19" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11">
-        <v>19</v>
-      </c>
-      <c r="B20" s="12" t="s">
+      <c r="A20" s="25">
+        <v>10019</v>
+      </c>
+      <c r="B20" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="29">
         <v>35344</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="28" t="s">
         <v>153</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="H20" s="14">
+      <c r="H20" s="30">
         <v>579253435499</v>
       </c>
-      <c r="I20" s="14" t="s">
+      <c r="I20" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="J20" s="14">
+      <c r="J20" s="30">
         <v>265104358643</v>
       </c>
-      <c r="K20" s="11" t="s">
+      <c r="K20" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L20" s="12" t="s">
+      <c r="L20" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M20" s="15" t="s">
+      <c r="M20" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N20" s="16">
+      <c r="N20" s="32">
         <v>22500</v>
       </c>
-      <c r="O20" s="16">
+      <c r="O20" s="32">
         <v>1500</v>
       </c>
-      <c r="P20" s="16">
+      <c r="P20" s="32">
         <v>500</v>
       </c>
-      <c r="Q20" s="16">
+      <c r="Q20" s="33">
         <v>500</v>
       </c>
-      <c r="R20" s="16">
+      <c r="R20" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S20" s="17">
+      <c r="S20" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T20" s="19" t="s">
-        <v>292</v>
-      </c>
-      <c r="U20" s="19" t="s">
-        <v>293</v>
-      </c>
-      <c r="V20" t="s">
-        <v>346</v>
-      </c>
-      <c r="W20" t="b">
+      <c r="T20" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="U20" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V20" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W20" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11">
-        <v>20</v>
-      </c>
-      <c r="B21" s="12" t="s">
+      <c r="A21" s="25">
+        <v>10020</v>
+      </c>
+      <c r="B21" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="29">
         <v>33281</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="H21" s="14">
+      <c r="H21" s="30">
         <v>399665157135</v>
       </c>
-      <c r="I21" s="14" t="s">
+      <c r="I21" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="J21" s="14">
+      <c r="J21" s="30">
         <v>260054585575</v>
       </c>
-      <c r="K21" s="11" t="s">
+      <c r="K21" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L21" s="12" t="s">
+      <c r="L21" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M21" s="15" t="s">
+      <c r="M21" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N21" s="16">
+      <c r="N21" s="32">
         <v>23250</v>
       </c>
-      <c r="O21" s="16">
+      <c r="O21" s="32">
         <v>1500</v>
       </c>
-      <c r="P21" s="16">
+      <c r="P21" s="32">
         <v>500</v>
       </c>
-      <c r="Q21" s="16">
+      <c r="Q21" s="33">
         <v>500</v>
       </c>
-      <c r="R21" s="16">
+      <c r="R21" s="32">
         <f t="shared" si="0"/>
         <v>11625</v>
       </c>
-      <c r="S21" s="17">
+      <c r="S21" s="27">
         <f t="shared" si="1"/>
         <v>138.39285714285714</v>
       </c>
-      <c r="T21" s="19" t="s">
-        <v>294</v>
-      </c>
-      <c r="U21" s="19" t="s">
-        <v>295</v>
-      </c>
-      <c r="V21" t="s">
-        <v>347</v>
-      </c>
-      <c r="W21" t="b">
+      <c r="T21" s="50" t="s">
+        <v>331</v>
+      </c>
+      <c r="U21" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V21" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W21" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11">
-        <v>21</v>
-      </c>
-      <c r="B22" s="12" t="s">
+      <c r="A22" s="25">
+        <v>10021</v>
+      </c>
+      <c r="B22" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="29">
         <v>31376</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="H22" s="14">
+      <c r="H22" s="30">
         <v>606386917510</v>
       </c>
-      <c r="I22" s="14" t="s">
+      <c r="I22" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="J22" s="14">
+      <c r="J22" s="30">
         <v>104907708845</v>
       </c>
-      <c r="K22" s="11" t="s">
+      <c r="K22" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L22" s="12" t="s">
+      <c r="L22" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M22" s="15" t="s">
+      <c r="M22" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N22" s="16">
+      <c r="N22" s="32">
         <v>23250</v>
       </c>
-      <c r="O22" s="16">
+      <c r="O22" s="32">
         <v>1500</v>
       </c>
-      <c r="P22" s="16">
+      <c r="P22" s="32">
         <v>500</v>
       </c>
-      <c r="Q22" s="16">
+      <c r="Q22" s="33">
         <v>500</v>
       </c>
-      <c r="R22" s="16">
+      <c r="R22" s="32">
         <f t="shared" si="0"/>
         <v>11625</v>
       </c>
-      <c r="S22" s="17">
+      <c r="S22" s="27">
         <f t="shared" si="1"/>
         <v>138.39285714285714</v>
       </c>
-      <c r="T22" s="19" t="s">
-        <v>296</v>
-      </c>
-      <c r="U22" s="19" t="s">
-        <v>297</v>
-      </c>
-      <c r="V22" t="s">
-        <v>348</v>
-      </c>
-      <c r="W22" t="b">
+      <c r="T22" s="50" t="s">
+        <v>332</v>
+      </c>
+      <c r="U22" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V22" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W22" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11">
-        <v>22</v>
-      </c>
-      <c r="B23" s="12" t="s">
+      <c r="A23" s="25">
+        <v>10022</v>
+      </c>
+      <c r="B23" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="29">
         <v>29277</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="H23" s="14">
+      <c r="H23" s="30">
         <v>357451271274</v>
       </c>
-      <c r="I23" s="14" t="s">
+      <c r="I23" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="J23" s="14">
+      <c r="J23" s="30">
         <v>113017988667</v>
       </c>
-      <c r="K23" s="11" t="s">
+      <c r="K23" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L23" s="12" t="s">
+      <c r="L23" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M23" s="15" t="s">
+      <c r="M23" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N23" s="16">
+      <c r="N23" s="32">
         <v>24000</v>
       </c>
-      <c r="O23" s="16">
+      <c r="O23" s="32">
         <v>1500</v>
       </c>
-      <c r="P23" s="16">
+      <c r="P23" s="32">
         <v>500</v>
       </c>
-      <c r="Q23" s="16">
+      <c r="Q23" s="33">
         <v>500</v>
       </c>
-      <c r="R23" s="16">
+      <c r="R23" s="32">
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="S23" s="17">
+      <c r="S23" s="27">
         <f t="shared" si="1"/>
         <v>142.85714285714286</v>
       </c>
-      <c r="T23" s="19" t="s">
-        <v>298</v>
-      </c>
-      <c r="U23" s="19" t="s">
-        <v>299</v>
-      </c>
-      <c r="V23" t="s">
-        <v>349</v>
-      </c>
-      <c r="W23" t="b">
+      <c r="T23" s="49" t="s">
+        <v>333</v>
+      </c>
+      <c r="U23" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V23" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W23" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11">
-        <v>23</v>
-      </c>
-      <c r="B24" s="12" t="s">
+      <c r="A24" s="25">
+        <v>10023</v>
+      </c>
+      <c r="B24" s="28" t="s">
         <v>176</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="28" t="s">
         <v>177</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="29">
         <v>30681</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="28" t="s">
         <v>178</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="H24" s="14">
+      <c r="H24" s="30">
         <v>548670482885</v>
       </c>
-      <c r="I24" s="14" t="s">
+      <c r="I24" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="J24" s="14">
+      <c r="J24" s="30">
         <v>360028104576</v>
       </c>
-      <c r="K24" s="11" t="s">
+      <c r="K24" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L24" s="12" t="s">
+      <c r="L24" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M24" s="15" t="s">
+      <c r="M24" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N24" s="16">
+      <c r="N24" s="32">
         <v>22500</v>
       </c>
-      <c r="O24" s="16">
+      <c r="O24" s="32">
         <v>1500</v>
       </c>
-      <c r="P24" s="16">
+      <c r="P24" s="32">
         <v>500</v>
       </c>
-      <c r="Q24" s="16">
+      <c r="Q24" s="33">
         <v>500</v>
       </c>
-      <c r="R24" s="16">
+      <c r="R24" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S24" s="17">
+      <c r="S24" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T24" s="19" t="s">
-        <v>300</v>
-      </c>
-      <c r="U24" s="19" t="s">
-        <v>301</v>
-      </c>
-      <c r="V24" t="s">
-        <v>350</v>
-      </c>
-      <c r="W24" t="b">
+      <c r="T24" s="50" t="s">
+        <v>334</v>
+      </c>
+      <c r="U24" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V24" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W24" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="11">
-        <v>24</v>
-      </c>
-      <c r="B25" s="12" t="s">
+      <c r="A25" s="25">
+        <v>10024</v>
+      </c>
+      <c r="B25" s="28" t="s">
         <v>182</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="28" t="s">
         <v>183</v>
       </c>
-      <c r="D25" s="13">
+      <c r="D25" s="29">
         <v>28842</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="28" t="s">
         <v>184</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="H25" s="14">
+      <c r="H25" s="30">
         <v>953901539995</v>
       </c>
-      <c r="I25" s="14" t="s">
+      <c r="I25" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="J25" s="14">
+      <c r="J25" s="30">
         <v>913108649964</v>
       </c>
-      <c r="K25" s="11" t="s">
+      <c r="K25" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L25" s="12" t="s">
+      <c r="L25" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M25" s="15" t="s">
+      <c r="M25" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="N25" s="16">
+      <c r="N25" s="32">
         <v>22500</v>
       </c>
-      <c r="O25" s="16">
+      <c r="O25" s="32">
         <v>1500</v>
       </c>
-      <c r="P25" s="16">
+      <c r="P25" s="32">
         <v>500</v>
       </c>
-      <c r="Q25" s="16">
+      <c r="Q25" s="33">
         <v>500</v>
       </c>
-      <c r="R25" s="16">
+      <c r="R25" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S25" s="17">
+      <c r="S25" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T25" s="19" t="s">
-        <v>302</v>
-      </c>
-      <c r="U25" s="19" t="s">
-        <v>303</v>
-      </c>
-      <c r="V25" t="s">
-        <v>351</v>
-      </c>
-      <c r="W25" t="b">
+      <c r="T25" s="49" t="s">
+        <v>284</v>
+      </c>
+      <c r="U25" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V25" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W25" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11">
-        <v>25</v>
-      </c>
-      <c r="B26" s="12" t="s">
+      <c r="A26" s="25">
+        <v>10025</v>
+      </c>
+      <c r="B26" s="28" t="s">
         <v>188</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="D26" s="13">
+      <c r="D26" s="29">
         <v>30821</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="E26" s="28" t="s">
         <v>190</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="H26" s="14">
+      <c r="H26" s="30">
         <v>753800654114</v>
       </c>
-      <c r="I26" s="14" t="s">
+      <c r="I26" s="30" t="s">
         <v>193</v>
       </c>
-      <c r="J26" s="14">
+      <c r="J26" s="30">
         <v>210546661243</v>
       </c>
-      <c r="K26" s="11" t="s">
+      <c r="K26" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L26" s="12" t="s">
+      <c r="L26" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M26" s="15" t="s">
+      <c r="M26" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N26" s="16">
+      <c r="N26" s="32">
         <v>24000</v>
       </c>
-      <c r="O26" s="16">
+      <c r="O26" s="32">
         <v>1500</v>
       </c>
-      <c r="P26" s="16">
+      <c r="P26" s="32">
         <v>500</v>
       </c>
-      <c r="Q26" s="16">
+      <c r="Q26" s="33">
         <v>500</v>
       </c>
-      <c r="R26" s="16">
+      <c r="R26" s="32">
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="S26" s="17">
+      <c r="S26" s="27">
         <f t="shared" si="1"/>
         <v>142.85714285714286</v>
       </c>
-      <c r="T26" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="U26" s="19" t="s">
-        <v>305</v>
-      </c>
-      <c r="V26" t="s">
-        <v>352</v>
-      </c>
-      <c r="W26" t="b">
+      <c r="T26" s="50" t="s">
+        <v>335</v>
+      </c>
+      <c r="U26" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V26" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W26" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="11">
-        <v>26</v>
-      </c>
-      <c r="B27" s="12" t="s">
+      <c r="A27" s="25">
+        <v>10026</v>
+      </c>
+      <c r="B27" s="28" t="s">
         <v>195</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="28" t="s">
         <v>196</v>
       </c>
-      <c r="D27" s="13">
+      <c r="D27" s="29">
         <v>25920</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="28" t="s">
         <v>197</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="F27" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="H27" s="14">
+      <c r="H27" s="30">
         <v>797639382265</v>
       </c>
-      <c r="I27" s="14" t="s">
+      <c r="I27" s="30" t="s">
         <v>200</v>
       </c>
-      <c r="J27" s="14">
+      <c r="J27" s="30">
         <v>210897095686</v>
       </c>
-      <c r="K27" s="11" t="s">
+      <c r="K27" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L27" s="12" t="s">
+      <c r="L27" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M27" s="15" t="s">
+      <c r="M27" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N27" s="16">
+      <c r="N27" s="32">
         <v>24750</v>
       </c>
-      <c r="O27" s="16">
+      <c r="O27" s="32">
         <v>1500</v>
       </c>
-      <c r="P27" s="16">
+      <c r="P27" s="32">
         <v>500</v>
       </c>
-      <c r="Q27" s="16">
+      <c r="Q27" s="33">
         <v>500</v>
       </c>
-      <c r="R27" s="16">
+      <c r="R27" s="32">
         <f t="shared" si="0"/>
         <v>12375</v>
       </c>
-      <c r="S27" s="17">
+      <c r="S27" s="27">
         <f t="shared" si="1"/>
         <v>147.32142857142858</v>
       </c>
-      <c r="T27" s="19" t="s">
-        <v>306</v>
-      </c>
-      <c r="U27" s="19" t="s">
-        <v>307</v>
-      </c>
-      <c r="V27" t="s">
-        <v>353</v>
-      </c>
-      <c r="W27" t="b">
+      <c r="T27" s="50" t="s">
+        <v>336</v>
+      </c>
+      <c r="U27" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V27" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W27" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="11">
-        <v>27</v>
-      </c>
-      <c r="B28" s="12" t="s">
+      <c r="A28" s="25">
+        <v>10027</v>
+      </c>
+      <c r="B28" s="28" t="s">
         <v>201</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="28" t="s">
         <v>202</v>
       </c>
-      <c r="D28" s="13">
+      <c r="D28" s="29">
         <v>31652</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="28" t="s">
         <v>203</v>
       </c>
-      <c r="F28" s="11" t="s">
+      <c r="F28" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G28" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="H28" s="14">
+      <c r="H28" s="30">
         <v>810909286264</v>
       </c>
-      <c r="I28" s="14" t="s">
+      <c r="I28" s="30" t="s">
         <v>206</v>
       </c>
-      <c r="J28" s="14">
+      <c r="J28" s="30">
         <v>211274476563</v>
       </c>
-      <c r="K28" s="11" t="s">
+      <c r="K28" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L28" s="12" t="s">
+      <c r="L28" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M28" s="15" t="s">
+      <c r="M28" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N28" s="16">
+      <c r="N28" s="32">
         <v>24750</v>
       </c>
-      <c r="O28" s="16">
+      <c r="O28" s="32">
         <v>1500</v>
       </c>
-      <c r="P28" s="16">
+      <c r="P28" s="32">
         <v>500</v>
       </c>
-      <c r="Q28" s="16">
+      <c r="Q28" s="33">
         <v>500</v>
       </c>
-      <c r="R28" s="16">
+      <c r="R28" s="32">
         <f t="shared" si="0"/>
         <v>12375</v>
       </c>
-      <c r="S28" s="17">
+      <c r="S28" s="27">
         <f t="shared" si="1"/>
         <v>147.32142857142858</v>
       </c>
-      <c r="T28" s="19" t="s">
-        <v>308</v>
-      </c>
-      <c r="U28" s="19" t="s">
-        <v>309</v>
-      </c>
-      <c r="V28" t="s">
-        <v>354</v>
-      </c>
-      <c r="W28" t="b">
+      <c r="T28" s="50" t="s">
+        <v>337</v>
+      </c>
+      <c r="U28" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V28" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W28" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11">
-        <v>28</v>
-      </c>
-      <c r="B29" s="12" t="s">
+      <c r="A29" s="25">
+        <v>10028</v>
+      </c>
+      <c r="B29" s="28" t="s">
         <v>207</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="28" t="s">
         <v>208</v>
       </c>
-      <c r="D29" s="13">
+      <c r="D29" s="29">
         <v>29932</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="28" t="s">
         <v>209</v>
       </c>
-      <c r="F29" s="11" t="s">
+      <c r="F29" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="H29" s="14">
+      <c r="H29" s="30">
         <v>934389652994</v>
       </c>
-      <c r="I29" s="14" t="s">
+      <c r="I29" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="J29" s="14">
+      <c r="J29" s="37">
         <v>122238077997</v>
       </c>
-      <c r="K29" s="11" t="s">
+      <c r="K29" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="L29" s="12" t="s">
+      <c r="L29" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M29" s="15" t="s">
+      <c r="M29" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N29" s="16">
+      <c r="N29" s="32">
         <v>24000</v>
       </c>
-      <c r="O29" s="16">
+      <c r="O29" s="32">
         <v>1500</v>
       </c>
-      <c r="P29" s="16">
+      <c r="P29" s="32">
         <v>500</v>
       </c>
-      <c r="Q29" s="16">
+      <c r="Q29" s="33">
         <v>500</v>
       </c>
-      <c r="R29" s="16">
+      <c r="R29" s="32">
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="S29" s="17">
+      <c r="S29" s="27">
         <f t="shared" si="1"/>
         <v>142.85714285714286</v>
       </c>
-      <c r="T29" s="19" t="s">
-        <v>310</v>
-      </c>
-      <c r="U29" s="19" t="s">
-        <v>311</v>
-      </c>
-      <c r="V29" t="s">
-        <v>355</v>
-      </c>
-      <c r="W29" t="b">
+      <c r="T29" s="50" t="s">
+        <v>338</v>
+      </c>
+      <c r="U29" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V29" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W29" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="11">
-        <v>29</v>
-      </c>
-      <c r="B30" s="12" t="s">
+      <c r="A30" s="25">
+        <v>10029</v>
+      </c>
+      <c r="B30" s="28" t="s">
         <v>213</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="28" t="s">
         <v>214</v>
       </c>
-      <c r="D30" s="13">
+      <c r="D30" s="29">
         <v>28722</v>
       </c>
-      <c r="E30" s="12" t="s">
+      <c r="E30" s="28" t="s">
         <v>215</v>
       </c>
-      <c r="F30" s="11" t="s">
+      <c r="F30" s="15" t="s">
         <v>216</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="H30" s="14">
+      <c r="H30" s="30">
         <v>351830469744</v>
       </c>
-      <c r="I30" s="14" t="s">
+      <c r="I30" s="44" t="s">
         <v>218</v>
       </c>
-      <c r="J30" s="14">
+      <c r="J30" s="19">
         <v>212141893454</v>
       </c>
-      <c r="K30" s="11" t="s">
+      <c r="K30" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="L30" s="12" t="s">
+      <c r="L30" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M30" s="15" t="s">
+      <c r="M30" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N30" s="16">
+      <c r="N30" s="32">
         <v>22500</v>
       </c>
-      <c r="O30" s="16">
+      <c r="O30" s="32">
         <v>1500</v>
       </c>
-      <c r="P30" s="16">
+      <c r="P30" s="32">
         <v>500</v>
       </c>
-      <c r="Q30" s="16">
+      <c r="Q30" s="33">
         <v>500</v>
       </c>
-      <c r="R30" s="16">
+      <c r="R30" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S30" s="17">
+      <c r="S30" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T30" s="19" t="s">
-        <v>312</v>
-      </c>
-      <c r="U30" s="19" t="s">
-        <v>313</v>
-      </c>
-      <c r="V30" t="s">
-        <v>356</v>
-      </c>
-      <c r="W30" t="b">
+      <c r="T30" s="50" t="s">
+        <v>339</v>
+      </c>
+      <c r="U30" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V30" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W30" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11">
-        <v>30</v>
-      </c>
-      <c r="B31" s="12" t="s">
+      <c r="A31" s="25">
+        <v>10030</v>
+      </c>
+      <c r="B31" s="28" t="s">
         <v>219</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="28" t="s">
         <v>220</v>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="29">
         <v>26768</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="28" t="s">
         <v>221</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="H31" s="14">
+      <c r="H31" s="30">
         <v>465087894112</v>
       </c>
-      <c r="I31" s="14" t="s">
+      <c r="I31" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="J31" s="14">
+      <c r="J31" s="19">
         <v>515012579765</v>
       </c>
-      <c r="K31" s="11" t="s">
+      <c r="K31" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="L31" s="12" t="s">
+      <c r="L31" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="M31" s="15" t="s">
+      <c r="M31" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N31" s="16">
+      <c r="N31" s="32">
         <v>22500</v>
       </c>
-      <c r="O31" s="16">
+      <c r="O31" s="32">
         <v>1500</v>
       </c>
-      <c r="P31" s="16">
+      <c r="P31" s="32">
         <v>500</v>
       </c>
-      <c r="Q31" s="16">
+      <c r="Q31" s="33">
         <v>500</v>
       </c>
-      <c r="R31" s="16">
+      <c r="R31" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S31" s="17">
+      <c r="S31" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T31" s="19" t="s">
-        <v>314</v>
-      </c>
-      <c r="U31" s="19" t="s">
-        <v>315</v>
-      </c>
-      <c r="V31" t="s">
-        <v>357</v>
-      </c>
-      <c r="W31" t="b">
+      <c r="T31" s="50" t="s">
+        <v>340</v>
+      </c>
+      <c r="U31" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V31" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W31" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11">
-        <v>31</v>
-      </c>
-      <c r="B32" s="12" t="s">
+      <c r="A32" s="25">
+        <v>10031</v>
+      </c>
+      <c r="B32" s="35" t="s">
         <v>225</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="35" t="s">
         <v>226</v>
       </c>
-      <c r="D32" s="13">
+      <c r="D32" s="36">
         <v>32535</v>
       </c>
-      <c r="E32" s="12" t="s">
+      <c r="E32" s="35" t="s">
         <v>227</v>
       </c>
-      <c r="F32" s="11" t="s">
+      <c r="F32" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="H32" s="14">
+      <c r="H32" s="37">
         <v>136451303068</v>
       </c>
-      <c r="I32" s="14" t="s">
+      <c r="I32" s="46" t="s">
         <v>230</v>
       </c>
-      <c r="J32" s="14">
+      <c r="J32" s="19">
         <v>110018813465</v>
       </c>
-      <c r="K32" s="11" t="s">
+      <c r="K32" s="47" t="s">
         <v>169</v>
       </c>
-      <c r="L32" s="12" t="s">
+      <c r="L32" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="M32" s="15" t="s">
+      <c r="M32" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="N32" s="16">
+      <c r="N32" s="48">
         <v>22500</v>
       </c>
-      <c r="O32" s="16">
+      <c r="O32" s="32">
         <v>1500</v>
       </c>
-      <c r="P32" s="16">
+      <c r="P32" s="32">
         <v>500</v>
       </c>
-      <c r="Q32" s="16">
+      <c r="Q32" s="33">
         <v>500</v>
       </c>
-      <c r="R32" s="16">
+      <c r="R32" s="32">
         <f t="shared" si="0"/>
         <v>11250</v>
       </c>
-      <c r="S32" s="17">
+      <c r="S32" s="27">
         <f t="shared" si="1"/>
         <v>133.92857142857142</v>
       </c>
-      <c r="T32" s="19" t="s">
-        <v>316</v>
-      </c>
-      <c r="U32" s="19" t="s">
-        <v>317</v>
-      </c>
-      <c r="V32" t="s">
-        <v>358</v>
-      </c>
-      <c r="W32" t="b">
+      <c r="T32" s="50" t="s">
+        <v>341</v>
+      </c>
+      <c r="U32" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V32" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="W32" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11">
-        <v>32</v>
-      </c>
-      <c r="B33" s="12" t="s">
+      <c r="A33" s="25">
+        <v>10032</v>
+      </c>
+      <c r="B33" s="28" t="s">
         <v>231</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="28" t="s">
         <v>232</v>
       </c>
-      <c r="D33" s="13">
+      <c r="D33" s="29">
         <v>33643</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="28" t="s">
         <v>233</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="H33" s="14">
+      <c r="H33" s="30">
         <v>601644902402</v>
       </c>
-      <c r="I33" s="14" t="s">
+      <c r="I33" s="44" t="s">
         <v>236</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="18">
         <v>697764069311</v>
       </c>
-      <c r="K33" s="11" t="s">
+      <c r="K33" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="L33" s="12" t="s">
+      <c r="L33" s="28" t="s">
         <v>237</v>
       </c>
-      <c r="M33" s="15" t="s">
+      <c r="M33" s="31" t="s">
         <v>238</v>
       </c>
-      <c r="N33" s="16">
+      <c r="N33" s="21">
         <v>52670</v>
       </c>
-      <c r="O33" s="16">
+      <c r="O33" s="32">
         <v>1500</v>
       </c>
-      <c r="P33" s="16">
+      <c r="P33" s="32">
         <v>1000</v>
       </c>
-      <c r="Q33" s="16">
+      <c r="Q33" s="33">
         <v>1000</v>
       </c>
-      <c r="R33" s="16">
+      <c r="R33" s="32">
         <f t="shared" si="0"/>
         <v>26335</v>
       </c>
-      <c r="S33" s="17">
+      <c r="S33" s="27">
         <f t="shared" si="1"/>
         <v>313.51190476190476</v>
       </c>
-      <c r="T33" s="19" t="s">
-        <v>318</v>
-      </c>
-      <c r="U33" s="19" t="s">
-        <v>319</v>
-      </c>
-      <c r="V33" t="s">
-        <v>359</v>
-      </c>
-      <c r="W33" t="b">
+      <c r="T33" s="49" t="s">
+        <v>285</v>
+      </c>
+      <c r="U33" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V33" s="49" t="s">
+        <v>286</v>
+      </c>
+      <c r="W33" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="11">
-        <v>33</v>
-      </c>
-      <c r="B34" s="12" t="s">
+      <c r="A34" s="25">
+        <v>10033</v>
+      </c>
+      <c r="B34" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="28" t="s">
         <v>239</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D34" s="29">
         <v>33193</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E34" s="28" t="s">
         <v>240</v>
       </c>
-      <c r="F34" s="11" t="s">
+      <c r="F34" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="G34" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="H34" s="14">
+      <c r="H34" s="30">
         <v>380685387212</v>
       </c>
-      <c r="I34" s="14" t="s">
+      <c r="I34" s="44" t="s">
         <v>243</v>
       </c>
-      <c r="J34" s="14">
+      <c r="J34" s="19">
         <v>993372963726</v>
       </c>
-      <c r="K34" s="11" t="s">
+      <c r="K34" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="L34" s="12" t="s">
+      <c r="L34" s="28" t="s">
         <v>244</v>
       </c>
-      <c r="M34" s="15" t="s">
+      <c r="M34" s="31" t="s">
         <v>238</v>
       </c>
-      <c r="N34" s="16">
+      <c r="N34" s="21">
         <v>52670</v>
       </c>
-      <c r="O34" s="16">
+      <c r="O34" s="32">
         <v>1500</v>
       </c>
-      <c r="P34" s="16">
+      <c r="P34" s="32">
         <v>1000</v>
       </c>
-      <c r="Q34" s="16">
+      <c r="Q34" s="33">
         <v>1000</v>
       </c>
-      <c r="R34" s="16">
+      <c r="R34" s="32">
         <f t="shared" si="0"/>
         <v>26335</v>
       </c>
-      <c r="S34" s="17">
+      <c r="S34" s="27">
         <f t="shared" si="1"/>
         <v>313.51190476190476</v>
       </c>
-      <c r="T34" s="19" t="s">
-        <v>320</v>
-      </c>
-      <c r="U34" s="19" t="s">
-        <v>321</v>
-      </c>
-      <c r="V34" t="s">
-        <v>360</v>
-      </c>
-      <c r="W34" t="b">
+      <c r="T34" s="49" t="s">
+        <v>287</v>
+      </c>
+      <c r="U34" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V34" s="49" t="s">
+        <v>288</v>
+      </c>
+      <c r="W34" s="50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="11">
-        <v>34</v>
-      </c>
-      <c r="B35" s="12" t="s">
+      <c r="A35" s="25">
+        <v>10034</v>
+      </c>
+      <c r="B35" s="28" t="s">
         <v>176</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="28" t="s">
         <v>245</v>
       </c>
-      <c r="D35" s="13">
+      <c r="D35" s="29">
         <v>33092</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="E35" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="F35" s="11" t="s">
+      <c r="F35" s="15" t="s">
         <v>247</v>
       </c>
-      <c r="G35" s="11" t="s">
+      <c r="G35" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="H35" s="14">
+      <c r="H35" s="30">
         <v>918460050077</v>
       </c>
-      <c r="I35" s="14" t="s">
+      <c r="I35" s="44" t="s">
         <v>249</v>
       </c>
-      <c r="J35" s="14">
+      <c r="J35" s="19">
         <v>874042259378</v>
       </c>
-      <c r="K35" s="11" t="s">
+      <c r="K35" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="L35" s="12" t="s">
+      <c r="L35" s="28" t="s">
         <v>250</v>
       </c>
-      <c r="M35" s="15" t="s">
+      <c r="M35" s="31" t="s">
         <v>238</v>
       </c>
-      <c r="N35" s="16">
+      <c r="N35" s="21">
         <v>52670</v>
       </c>
-      <c r="O35" s="16">
+      <c r="O35" s="32">
         <v>1500</v>
       </c>
-      <c r="P35" s="16">
+      <c r="P35" s="32">
         <v>1000</v>
       </c>
-      <c r="Q35" s="16">
+      <c r="Q35" s="33">
         <v>1000</v>
       </c>
-      <c r="R35" s="16">
+      <c r="R35" s="32">
         <f t="shared" si="0"/>
         <v>26335</v>
       </c>
-      <c r="S35" s="17">
+      <c r="S35" s="27">
         <f t="shared" si="1"/>
         <v>313.51190476190476</v>
       </c>
-      <c r="T35" s="19" t="s">
-        <v>322</v>
-      </c>
-      <c r="U35" s="19" t="s">
-        <v>323</v>
-      </c>
-      <c r="V35" t="s">
-        <v>361</v>
-      </c>
-      <c r="W35" t="b">
+      <c r="T35" s="50" t="s">
+        <v>267</v>
+      </c>
+      <c r="U35" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="V35" s="49" t="s">
+        <v>289</v>
+      </c>
+      <c r="W35" s="50" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4109,6 +4238,407 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D891F36-386F-4E1A-8E0A-C1E924593AAA}">
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="23" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>290</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>291</v>
+      </c>
+      <c r="C3" s="49" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="B4" s="49" t="s">
+        <v>292</v>
+      </c>
+      <c r="C4" s="49" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>259</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>293</v>
+      </c>
+      <c r="C5" s="49" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>294</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="23" t="s">
+        <v>276</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>295</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="23" t="s">
+        <v>324</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>261</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>296</v>
+      </c>
+      <c r="C9" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>325</v>
+      </c>
+      <c r="B10" s="49" t="s">
+        <v>307</v>
+      </c>
+      <c r="C10" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>262</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>297</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>263</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>298</v>
+      </c>
+      <c r="C12" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>326</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>308</v>
+      </c>
+      <c r="C13" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>264</v>
+      </c>
+      <c r="B14" s="49" t="s">
+        <v>299</v>
+      </c>
+      <c r="C14" s="49" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>265</v>
+      </c>
+      <c r="B15" s="49" t="s">
+        <v>300</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>327</v>
+      </c>
+      <c r="B16" s="49" t="s">
+        <v>309</v>
+      </c>
+      <c r="C16" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>266</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>301</v>
+      </c>
+      <c r="C17" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="23" t="s">
+        <v>328</v>
+      </c>
+      <c r="B18" s="49" t="s">
+        <v>310</v>
+      </c>
+      <c r="C18" s="49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="C19" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>330</v>
+      </c>
+      <c r="B20" s="49" t="s">
+        <v>312</v>
+      </c>
+      <c r="C20" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>331</v>
+      </c>
+      <c r="B21" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>332</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>314</v>
+      </c>
+      <c r="C22" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="23" t="s">
+        <v>333</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>315</v>
+      </c>
+      <c r="C23" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>334</v>
+      </c>
+      <c r="B24" s="49" t="s">
+        <v>316</v>
+      </c>
+      <c r="C24" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="B25" s="49" t="s">
+        <v>302</v>
+      </c>
+      <c r="C25" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>335</v>
+      </c>
+      <c r="B26" s="49" t="s">
+        <v>317</v>
+      </c>
+      <c r="C26" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>336</v>
+      </c>
+      <c r="B27" s="49" t="s">
+        <v>318</v>
+      </c>
+      <c r="C27" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>337</v>
+      </c>
+      <c r="B28" s="49" t="s">
+        <v>319</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>338</v>
+      </c>
+      <c r="B29" s="49" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>339</v>
+      </c>
+      <c r="B30" s="49" t="s">
+        <v>321</v>
+      </c>
+      <c r="C30" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>340</v>
+      </c>
+      <c r="B31" s="49" t="s">
+        <v>322</v>
+      </c>
+      <c r="C31" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>341</v>
+      </c>
+      <c r="B32" s="49" t="s">
+        <v>323</v>
+      </c>
+      <c r="C32" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="23" t="s">
+        <v>285</v>
+      </c>
+      <c r="B33" s="49" t="s">
+        <v>303</v>
+      </c>
+      <c r="C33" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="23" t="s">
+        <v>287</v>
+      </c>
+      <c r="B34" s="49" t="s">
+        <v>304</v>
+      </c>
+      <c r="C34" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B35" s="49" t="s">
+        <v>305</v>
+      </c>
+      <c r="C35" s="49" t="s">
+        <v>279</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C35" xr:uid="{9D891F36-386F-4E1A-8E0A-C1E924593AAA}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F2176"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>